<commit_message>
Integrate conferences into publications
</commit_message>
<xml_diff>
--- a/PhD_PI_Listup.xlsx
+++ b/PhD_PI_Listup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hyeonbeen/Git/LaTeX-Docs/MyResume/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D707683-0E5B-9F48-A192-AEE8C9A0360F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1BEB974-4D3A-2044-B5E8-A1B5D4BE715B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="22540" activeTab="4" xr2:uid="{422F52E5-BD25-DB4D-B83C-2D9AD22AB820}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="22540" xr2:uid="{422F52E5-BD25-DB4D-B83C-2D9AD22AB820}"/>
   </bookViews>
   <sheets>
     <sheet name="Professors" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2352" uniqueCount="768">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2389" uniqueCount="783">
   <si>
     <t>PI</t>
   </si>
@@ -2440,9 +2440,6 @@
     <t>Control theory, Learning little, lots of robots</t>
   </si>
   <si>
-    <t>Note</t>
-  </si>
-  <si>
     <t>Supplementary form (500w)</t>
   </si>
   <si>
@@ -2510,9 +2507,6 @@
     <t>(SOP==PS, ~2p)</t>
   </si>
   <si>
-    <t>Additional Coursework</t>
-  </si>
-  <si>
     <t>(SOP==PS ~2p, +Community), +(Community 200w)</t>
   </si>
   <si>
@@ -2546,19 +2540,70 @@
     <t>LoR, TOEFL after deadline?</t>
   </si>
   <si>
-    <t>LoR받고 제출만</t>
-  </si>
-  <si>
-    <t>Video, LoR받고 제출만</t>
-  </si>
-  <si>
     <t>Ann Majewicz Fey</t>
   </si>
   <si>
     <t>Mitchell W Pryor</t>
   </si>
   <si>
-    <t>Submitted, awaiting MyStatus</t>
+    <t>Accept LoR after deadline, TOEFL within deadline</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>In progress, LoR</t>
+  </si>
+  <si>
+    <t>Submitted, LoR</t>
+  </si>
+  <si>
+    <t>In progress</t>
+  </si>
+  <si>
+    <t>AeroAstro</t>
+  </si>
+  <si>
+    <t>Marco Pavone</t>
+  </si>
+  <si>
+    <t>Physically grounded robot planning, physics-based digital twin, data-driven control</t>
+  </si>
+  <si>
+    <t>Safe AI, HJ reachability, MPC, Physics-informed ML, Safety guided IL</t>
+  </si>
+  <si>
+    <t>Somil Bansal</t>
+  </si>
+  <si>
+    <t>Safe AI, Navigation &amp; SLAM, sensor fusion</t>
+  </si>
+  <si>
+    <t>Grace Gao</t>
+  </si>
+  <si>
+    <t>AeroAstro, CS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Decision making in uncertainty, Safe AI, Navigation, Adaptive sampling, Constrained and domain-informed policy, </t>
+  </si>
+  <si>
+    <t>Mykel Kochenderfer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Multi-agent robots, vision-based perception, Geometry-embedded, differntiable simulator, </t>
+  </si>
+  <si>
+    <t>after admission</t>
+  </si>
+  <si>
+    <t>we accept students</t>
+  </si>
+  <si>
+    <t>Mac Schwager</t>
+  </si>
+  <si>
+    <t>AeroAstro, EE</t>
   </si>
 </sst>
 </file>
@@ -2974,10 +3019,10 @@
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -3315,7 +3360,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{132F7052-85E4-E84F-9E71-39A4BFB15A06}">
-  <dimension ref="A1:H177"/>
+  <dimension ref="A1:H182"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.5" style="5" bestFit="1" customWidth="1"/>
@@ -4000,10 +4045,10 @@
         <v>86</v>
       </c>
       <c r="C35" s="6" t="s">
+        <v>745</v>
+      </c>
+      <c r="F35" s="6" t="s">
         <v>746</v>
-      </c>
-      <c r="F35" s="6" t="s">
-        <v>747</v>
       </c>
     </row>
     <row r="36" spans="1:6" s="70" customFormat="1" x14ac:dyDescent="0.2">
@@ -4014,10 +4059,10 @@
         <v>86</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.2">
@@ -4684,10 +4729,10 @@
         <v>8</v>
       </c>
       <c r="C74" s="17" t="s">
-        <v>753</v>
+        <v>751</v>
       </c>
       <c r="D74" s="16" t="s">
-        <v>754</v>
+        <v>752</v>
       </c>
       <c r="E74" s="16" t="s">
         <v>128</v>
@@ -4704,10 +4749,10 @@
         <v>8</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>758</v>
+        <v>756</v>
       </c>
       <c r="D75" s="70" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
       <c r="E75" s="70" t="s">
         <v>28</v>
@@ -4724,16 +4769,16 @@
         <v>8</v>
       </c>
       <c r="C76" s="13" t="s">
-        <v>756</v>
+        <v>754</v>
       </c>
       <c r="D76" s="12" t="s">
-        <v>755</v>
+        <v>753</v>
       </c>
       <c r="E76" s="12" t="s">
         <v>29</v>
       </c>
       <c r="F76" s="6" t="s">
-        <v>757</v>
+        <v>755</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.2">
@@ -6621,12 +6666,97 @@
         <v>718</v>
       </c>
     </row>
-    <row r="177" spans="3:6" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:6" x14ac:dyDescent="0.2">
       <c r="C177" s="3" t="s">
         <v>721</v>
       </c>
       <c r="F177" s="3" t="s">
         <v>720</v>
+      </c>
+    </row>
+    <row r="178" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A178" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B178" s="1" t="s">
+        <v>768</v>
+      </c>
+      <c r="C178" s="3" t="s">
+        <v>769</v>
+      </c>
+      <c r="D178" s="1" t="s">
+        <v>770</v>
+      </c>
+      <c r="E178" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F178" s="3" t="s">
+        <v>779</v>
+      </c>
+    </row>
+    <row r="179" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B179" s="1" t="s">
+        <v>768</v>
+      </c>
+      <c r="C179" s="3" t="s">
+        <v>772</v>
+      </c>
+      <c r="D179" s="1" t="s">
+        <v>771</v>
+      </c>
+      <c r="E179" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="F179" s="3" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="180" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B180" s="1" t="s">
+        <v>782</v>
+      </c>
+      <c r="C180" s="3" t="s">
+        <v>774</v>
+      </c>
+      <c r="D180" s="1" t="s">
+        <v>773</v>
+      </c>
+      <c r="E180" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="F180" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="181" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B181" s="1" t="s">
+        <v>775</v>
+      </c>
+      <c r="C181" s="3" t="s">
+        <v>777</v>
+      </c>
+      <c r="D181" s="1" t="s">
+        <v>776</v>
+      </c>
+      <c r="E181" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F181" s="3" t="s">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="182" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B182" s="1" t="s">
+        <v>768</v>
+      </c>
+      <c r="C182" s="3" t="s">
+        <v>781</v>
+      </c>
+      <c r="D182" s="1" t="s">
+        <v>778</v>
+      </c>
+      <c r="E182" s="1" t="s">
+        <v>128</v>
       </c>
     </row>
   </sheetData>
@@ -6920,6 +7050,15 @@
     <hyperlink ref="C76" r:id="rId286" xr:uid="{9A5DB3D4-9E7F-4E4F-8FD1-1C53D9174029}"/>
     <hyperlink ref="F76" r:id="rId287" display="Yes" xr:uid="{2DFC89E2-23AF-E34C-8638-EF037FE8110A}"/>
     <hyperlink ref="F75" r:id="rId288" xr:uid="{9467102C-D9A3-D34D-8F48-BC279E982807}"/>
+    <hyperlink ref="C178" r:id="rId289" xr:uid="{03171C12-4519-3B41-A03E-DE3C397082EB}"/>
+    <hyperlink ref="C179" r:id="rId290" display="https://smlbansal.github.io/sia-lab/publications.html" xr:uid="{650F4A89-D858-CA4B-B4A6-B79D1A57D72C}"/>
+    <hyperlink ref="C180" r:id="rId291" xr:uid="{0D692EF2-94EF-B041-8E80-651E8BC65D8C}"/>
+    <hyperlink ref="C181" r:id="rId292" display="https://sisl.stanford.edu/publications/" xr:uid="{A6A553D8-9382-9E49-8240-B67BB7BAC09C}"/>
+    <hyperlink ref="C182" r:id="rId293" display="https://msl.stanford.edu/" xr:uid="{FB3B84C8-DC14-A94A-93B3-7406F17A9333}"/>
+    <hyperlink ref="F179" r:id="rId294" xr:uid="{B6C3342E-C53D-DD46-9391-94C758679435}"/>
+    <hyperlink ref="F180" r:id="rId295" xr:uid="{D210D5B9-A70F-3146-AE86-502C97F3E44D}"/>
+    <hyperlink ref="F178" r:id="rId296" display="I'll try best to respond" xr:uid="{37695FF8-F824-3D47-93CE-5D6F335DF153}"/>
+    <hyperlink ref="F181" r:id="rId297" xr:uid="{AAB6B7F7-C053-E343-A6A4-58E240818AAB}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -11145,13 +11284,13 @@
     <col min="2" max="2" width="17.33203125" style="5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.1640625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.33203125" style="9" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="35.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="73.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="40.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="29.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12" style="11" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="41.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="29.1640625" style="1" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="7.83203125" style="11" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="19.5" style="1" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="20.33203125" style="1" bestFit="1" customWidth="1"/>
@@ -11172,8 +11311,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A1" s="5" t="s">
-        <v>732</v>
+      <c r="A1" s="4" t="s">
+        <v>764</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>3</v>
@@ -11200,7 +11339,7 @@
         <v>199</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>762</v>
+        <v>760</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>219</v>
@@ -11246,67 +11385,43 @@
       </c>
     </row>
     <row r="2" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="B2" s="69" t="s">
+      <c r="A2" s="1" t="s">
+        <v>767</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="6" t="s">
-        <v>8</v>
+      <c r="C2" s="3" t="s">
+        <v>768</v>
       </c>
       <c r="D2" s="70" t="s">
-        <v>317</v>
-      </c>
-      <c r="E2" s="63">
+        <v>327</v>
+      </c>
+      <c r="E2" s="62">
         <v>45993</v>
       </c>
-      <c r="F2" s="70" t="s">
+      <c r="F2" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="G2" s="70" t="s">
+      <c r="G2" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="H2" s="70" t="s">
-        <v>733</v>
-      </c>
-      <c r="I2" s="71">
+      <c r="I2" s="11">
         <v>125</v>
       </c>
-      <c r="J2" s="70" t="s">
-        <v>205</v>
-      </c>
-      <c r="K2" s="26" t="s">
-        <v>221</v>
-      </c>
-      <c r="L2" s="44" t="s">
-        <v>508</v>
-      </c>
-      <c r="M2" s="7" t="s">
-        <v>640</v>
-      </c>
-      <c r="N2" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="O2" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="P2" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="Q2" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="R2" s="3" t="s">
-        <v>9</v>
+      <c r="J2" s="1" t="s">
+        <v>207</v>
       </c>
       <c r="T2" s="1" t="s">
         <v>597</v>
       </c>
-      <c r="V2" s="70" t="s">
-        <v>206</v>
-      </c>
-      <c r="W2" s="70">
+      <c r="V2" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="W2" s="1">
         <v>4704</v>
       </c>
-      <c r="X2" s="70" t="s">
+      <c r="X2" s="1" t="s">
         <v>597</v>
       </c>
     </row>
@@ -11390,7 +11505,7 @@
         <v>384</v>
       </c>
       <c r="H4" s="70" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="I4" s="71">
         <v>105</v>
@@ -11437,6 +11552,9 @@
       </c>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>765</v>
+      </c>
       <c r="B5" s="69" t="s">
         <v>97</v>
       </c>
@@ -11454,13 +11572,13 @@
         <v>243</v>
       </c>
       <c r="H5" s="27" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="I5" s="71">
         <v>90</v>
       </c>
-      <c r="J5" s="70" t="s">
-        <v>275</v>
+      <c r="J5" s="27" t="s">
+        <v>763</v>
       </c>
       <c r="K5" s="44" t="s">
         <v>286</v>
@@ -11471,7 +11589,7 @@
       <c r="M5" s="7" t="s">
         <v>643</v>
       </c>
-      <c r="N5" s="13" t="s">
+      <c r="N5" s="45" t="s">
         <v>107</v>
       </c>
       <c r="O5" s="45" t="s">
@@ -11558,7 +11676,7 @@
       <c r="B7" s="69" t="s">
         <v>78</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="27" t="s">
         <v>65</v>
       </c>
       <c r="D7" s="70" t="s">
@@ -11572,31 +11690,31 @@
         <v>201</v>
       </c>
       <c r="H7" s="70" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="I7" s="71">
         <v>90</v>
       </c>
       <c r="J7" s="70"/>
-      <c r="K7" s="26" t="s">
+      <c r="K7" s="44" t="s">
         <v>236</v>
       </c>
       <c r="L7" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="M7" s="3" t="s">
+      <c r="M7" s="7" t="s">
         <v>723</v>
       </c>
-      <c r="N7" s="13" t="s">
+      <c r="N7" s="45" t="s">
         <v>79</v>
       </c>
-      <c r="O7" s="20" t="s">
+      <c r="O7" s="28" t="s">
         <v>373</v>
       </c>
       <c r="T7" s="1" t="s">
         <v>597</v>
       </c>
-      <c r="V7" s="6" t="s">
+      <c r="V7" s="27" t="s">
         <v>354</v>
       </c>
       <c r="W7" s="70">
@@ -11610,7 +11728,7 @@
       <c r="B8" s="69" t="s">
         <v>109</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="27" t="s">
         <v>86</v>
       </c>
       <c r="D8" s="70" t="s">
@@ -11624,7 +11742,7 @@
         <v>638</v>
       </c>
       <c r="H8" s="70" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="I8" s="71">
         <v>105</v>
@@ -11663,7 +11781,7 @@
       <c r="B9" s="69" t="s">
         <v>374</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="27" t="s">
         <v>92</v>
       </c>
       <c r="D9" s="70" t="s">
@@ -11678,8 +11796,8 @@
       <c r="G9" s="70" t="s">
         <v>201</v>
       </c>
-      <c r="H9" s="6" t="s">
-        <v>738</v>
+      <c r="H9" s="27" t="s">
+        <v>737</v>
       </c>
       <c r="I9" s="71">
         <v>90</v>
@@ -11693,16 +11811,16 @@
       <c r="L9" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="M9" s="3" t="s">
+      <c r="M9" s="7" t="s">
         <v>724</v>
       </c>
-      <c r="N9" s="6" t="s">
+      <c r="N9" s="27" t="s">
         <v>380</v>
       </c>
-      <c r="O9" s="13" t="s">
+      <c r="O9" s="45" t="s">
         <v>377</v>
       </c>
-      <c r="P9" s="29" t="s">
+      <c r="P9" s="78" t="s">
         <v>375</v>
       </c>
       <c r="T9" s="1" t="s">
@@ -11779,7 +11897,7 @@
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="B11" s="69" t="s">
         <v>82</v>
@@ -11817,16 +11935,16 @@
       <c r="O11" s="67" t="s">
         <v>537</v>
       </c>
-      <c r="P11" s="3" t="s">
-        <v>765</v>
-      </c>
-      <c r="Q11" s="3" t="s">
-        <v>766</v>
+      <c r="P11" s="7" t="s">
+        <v>761</v>
+      </c>
+      <c r="Q11" s="7" t="s">
+        <v>762</v>
       </c>
       <c r="R11" s="28" t="s">
         <v>535</v>
       </c>
-      <c r="S11" s="3"/>
+      <c r="S11" s="7"/>
       <c r="T11" s="1" t="s">
         <v>597</v>
       </c>
@@ -11917,7 +12035,7 @@
         <v>296</v>
       </c>
       <c r="H13" s="27" t="s">
-        <v>752</v>
+        <v>750</v>
       </c>
       <c r="I13" s="71">
         <v>90</v>
@@ -11963,7 +12081,7 @@
       <c r="B14" s="69" t="s">
         <v>133</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="27" t="s">
         <v>8</v>
       </c>
       <c r="D14" s="70" t="s">
@@ -11973,11 +12091,11 @@
         <v>46006</v>
       </c>
       <c r="F14" s="70"/>
-      <c r="G14" s="6" t="s">
+      <c r="G14" s="27" t="s">
         <v>201</v>
       </c>
       <c r="H14" s="27" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="I14" s="71">
         <v>85</v>
@@ -11994,16 +12112,16 @@
       <c r="M14" s="7" t="s">
         <v>649</v>
       </c>
-      <c r="N14" s="13" t="s">
+      <c r="N14" s="45" t="s">
         <v>136</v>
       </c>
-      <c r="O14" s="13" t="s">
+      <c r="O14" s="45" t="s">
         <v>305</v>
       </c>
       <c r="T14" s="1" t="s">
         <v>597</v>
       </c>
-      <c r="V14" s="6" t="s">
+      <c r="V14" s="27" t="s">
         <v>294</v>
       </c>
       <c r="W14" s="70">
@@ -12015,12 +12133,12 @@
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>763</v>
+        <v>765</v>
       </c>
       <c r="B15" s="69" t="s">
         <v>60</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="27" t="s">
         <v>8</v>
       </c>
       <c r="D15" s="70" t="s">
@@ -12034,39 +12152,39 @@
         <v>201</v>
       </c>
       <c r="H15" s="70" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="I15" s="71">
         <v>60</v>
       </c>
-      <c r="J15" s="6" t="s">
+      <c r="J15" s="27" t="s">
         <v>271</v>
       </c>
-      <c r="K15" s="26" t="s">
+      <c r="K15" s="44" t="s">
         <v>590</v>
       </c>
       <c r="L15" s="44" t="s">
         <v>29</v>
       </c>
-      <c r="M15" s="3" t="s">
+      <c r="M15" s="7" t="s">
         <v>725</v>
       </c>
-      <c r="N15" s="13" t="s">
+      <c r="N15" s="45" t="s">
+        <v>754</v>
+      </c>
+      <c r="O15" s="45" t="s">
+        <v>67</v>
+      </c>
+      <c r="P15" s="48" t="s">
+        <v>751</v>
+      </c>
+      <c r="Q15" s="48" t="s">
         <v>756</v>
       </c>
-      <c r="O15" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="P15" s="17" t="s">
-        <v>753</v>
-      </c>
-      <c r="Q15" s="17" t="s">
-        <v>758</v>
-      </c>
-      <c r="R15" s="20" t="s">
+      <c r="R15" s="28" t="s">
         <v>61</v>
       </c>
-      <c r="S15" s="6"/>
+      <c r="S15" s="27"/>
       <c r="T15" s="1" t="s">
         <v>597</v>
       </c>
@@ -12100,7 +12218,7 @@
         <v>201</v>
       </c>
       <c r="H16" s="27" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="I16" s="71">
         <v>105</v>
@@ -12154,7 +12272,7 @@
         <v>201</v>
       </c>
       <c r="H17" s="27" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="I17" s="71">
         <v>105</v>
@@ -12193,13 +12311,13 @@
       <c r="B18" s="69" t="s">
         <v>414</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C18" s="27" t="s">
         <v>8</v>
       </c>
       <c r="D18" s="70" t="s">
         <v>323</v>
       </c>
-      <c r="E18" s="77">
+      <c r="E18" s="76">
         <v>46007</v>
       </c>
       <c r="F18" s="70" t="s">
@@ -12215,26 +12333,26 @@
         <v>95</v>
       </c>
       <c r="J18" s="71"/>
-      <c r="K18" s="6" t="s">
+      <c r="K18" s="27" t="s">
         <v>590</v>
       </c>
       <c r="L18" s="1"/>
-      <c r="N18" s="29" t="s">
+      <c r="N18" s="78" t="s">
         <v>415</v>
       </c>
-      <c r="O18" s="3" t="s">
+      <c r="O18" s="7" t="s">
         <v>472</v>
       </c>
-      <c r="P18" s="3" t="s">
+      <c r="P18" s="7" t="s">
         <v>474</v>
       </c>
-      <c r="Q18" s="3" t="s">
+      <c r="Q18" s="7" t="s">
         <v>470</v>
       </c>
       <c r="T18" s="1" t="s">
         <v>597</v>
       </c>
-      <c r="V18" s="6" t="s">
+      <c r="V18" s="27" t="s">
         <v>208</v>
       </c>
       <c r="W18" s="70">
@@ -12246,7 +12364,7 @@
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
-        <v>764</v>
+        <v>765</v>
       </c>
       <c r="B19" s="69" t="s">
         <v>628</v>
@@ -12265,7 +12383,7 @@
         <v>201</v>
       </c>
       <c r="H19" s="27" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="I19" s="71" t="s">
         <v>698</v>
@@ -12284,7 +12402,7 @@
       <c r="O19" s="48" t="s">
         <v>170</v>
       </c>
-      <c r="P19" s="6" t="s">
+      <c r="P19" s="27" t="s">
         <v>730</v>
       </c>
       <c r="T19" s="1" t="s">
@@ -12301,29 +12419,26 @@
       </c>
     </row>
     <row r="20" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A20" s="1" t="s">
-        <v>751</v>
-      </c>
       <c r="B20" s="69" t="s">
         <v>342</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="27" t="s">
         <v>8</v>
       </c>
       <c r="D20" s="70" t="s">
         <v>324</v>
       </c>
-      <c r="E20" s="77">
+      <c r="E20" s="76">
         <v>46006</v>
       </c>
       <c r="F20" s="70" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="G20" s="70" t="s">
         <v>201</v>
       </c>
       <c r="H20" s="27" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="I20" s="71">
         <v>80</v>
@@ -12359,12 +12474,12 @@
     </row>
     <row r="21" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>759</v>
+        <v>757</v>
       </c>
       <c r="B21" s="5" t="s">
         <v>599</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" s="27" t="s">
         <v>353</v>
       </c>
       <c r="D21" s="1" t="s">
@@ -12387,88 +12502,33 @@
         <v>29</v>
       </c>
       <c r="L21" s="1"/>
-      <c r="N21" s="17" t="s">
+      <c r="N21" s="48" t="s">
         <v>192</v>
       </c>
-      <c r="O21" s="17" t="s">
+      <c r="O21" s="48" t="s">
         <v>195</v>
       </c>
-      <c r="P21" s="3" t="s">
+      <c r="P21" s="7" t="s">
         <v>190</v>
       </c>
       <c r="T21" s="34" t="s">
-        <v>760</v>
-      </c>
-      <c r="V21" s="6" t="s">
+        <v>758</v>
+      </c>
+      <c r="V21" s="27" t="s">
         <v>208</v>
       </c>
       <c r="W21" s="1" t="s">
         <v>357</v>
       </c>
       <c r="X21" s="34" t="s">
-        <v>760</v>
+        <v>758</v>
       </c>
     </row>
     <row r="22" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="I22" s="11"/>
-      <c r="J22" s="1"/>
-      <c r="K22" s="1"/>
       <c r="L22" s="1"/>
     </row>
     <row r="23" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="I23" s="11"/>
-      <c r="J23" s="1"/>
-      <c r="K23" s="1"/>
       <c r="L23" s="1"/>
-    </row>
-    <row r="24" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="B24" s="69" t="s">
-        <v>4</v>
-      </c>
-      <c r="C24" s="27" t="s">
-        <v>5</v>
-      </c>
-      <c r="D24" s="70" t="s">
-        <v>327</v>
-      </c>
-      <c r="E24" s="25">
-        <v>45992</v>
-      </c>
-      <c r="F24" s="70"/>
-      <c r="G24" s="70" t="s">
-        <v>201</v>
-      </c>
-      <c r="H24" s="70" t="s">
-        <v>203</v>
-      </c>
-      <c r="I24" s="71">
-        <v>125</v>
-      </c>
-      <c r="J24" s="70" t="s">
-        <v>205</v>
-      </c>
-      <c r="K24" s="44" t="s">
-        <v>220</v>
-      </c>
-      <c r="L24" s="44"/>
-      <c r="M24" s="7" t="s">
-        <v>640</v>
-      </c>
-      <c r="N24" s="45" t="s">
-        <v>6</v>
-      </c>
-      <c r="O24" s="68" t="s">
-        <v>510</v>
-      </c>
-      <c r="V24" s="70" t="s">
-        <v>206</v>
-      </c>
-      <c r="W24" s="70">
-        <v>4704</v>
-      </c>
-      <c r="X24" s="70" t="s">
-        <v>597</v>
-      </c>
     </row>
     <row r="25" spans="1:24" x14ac:dyDescent="0.2">
       <c r="B25" s="69" t="s">
@@ -12583,7 +12643,7 @@
         <v>201</v>
       </c>
       <c r="H27" s="66" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="I27" s="71">
         <v>80</v>
@@ -12631,11 +12691,11 @@
         <v>46006</v>
       </c>
       <c r="F28" s="70"/>
-      <c r="G28" s="78" t="s">
+      <c r="G28" s="77" t="s">
         <v>621</v>
       </c>
       <c r="H28" s="70" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="I28" s="71">
         <v>85</v>
@@ -12676,58 +12736,150 @@
       </c>
     </row>
     <row r="29" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="I29" s="11"/>
-      <c r="J29" s="1"/>
-      <c r="K29" s="1"/>
-      <c r="L29" s="1"/>
+      <c r="B29" s="69" t="s">
+        <v>4</v>
+      </c>
+      <c r="C29" s="27" t="s">
+        <v>8</v>
+      </c>
+      <c r="D29" s="70" t="s">
+        <v>317</v>
+      </c>
+      <c r="E29" s="63">
+        <v>45993</v>
+      </c>
+      <c r="F29" s="70" t="s">
+        <v>269</v>
+      </c>
+      <c r="G29" s="70" t="s">
+        <v>201</v>
+      </c>
+      <c r="H29" s="70" t="s">
+        <v>732</v>
+      </c>
+      <c r="I29" s="71">
+        <v>125</v>
+      </c>
+      <c r="J29" s="70" t="s">
+        <v>205</v>
+      </c>
+      <c r="K29" s="44" t="s">
+        <v>221</v>
+      </c>
+      <c r="L29" s="44" t="s">
+        <v>508</v>
+      </c>
+      <c r="M29" s="7" t="s">
+        <v>640</v>
+      </c>
+      <c r="N29" s="45" t="s">
+        <v>15</v>
+      </c>
+      <c r="O29" s="45" t="s">
+        <v>23</v>
+      </c>
+      <c r="P29" s="45" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q29" s="45" t="s">
+        <v>17</v>
+      </c>
+      <c r="R29" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="T29" s="1" t="s">
+        <v>597</v>
+      </c>
+      <c r="V29" s="70" t="s">
+        <v>206</v>
+      </c>
+      <c r="W29" s="70">
+        <v>4704</v>
+      </c>
+      <c r="X29" s="70" t="s">
+        <v>597</v>
+      </c>
     </row>
     <row r="30" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="I30" s="11"/>
-      <c r="J30" s="1"/>
-      <c r="K30" s="1"/>
-      <c r="L30" s="1"/>
+      <c r="A30" s="1" t="s">
+        <v>767</v>
+      </c>
+      <c r="B30" s="69" t="s">
+        <v>4</v>
+      </c>
+      <c r="C30" s="27" t="s">
+        <v>5</v>
+      </c>
+      <c r="D30" s="70" t="s">
+        <v>327</v>
+      </c>
+      <c r="E30" s="63">
+        <v>45992</v>
+      </c>
+      <c r="F30" s="70" t="s">
+        <v>269</v>
+      </c>
+      <c r="G30" s="70" t="s">
+        <v>201</v>
+      </c>
+      <c r="H30" s="70" t="s">
+        <v>203</v>
+      </c>
+      <c r="I30" s="71">
+        <v>125</v>
+      </c>
+      <c r="J30" s="70" t="s">
+        <v>205</v>
+      </c>
+      <c r="K30" s="44" t="s">
+        <v>220</v>
+      </c>
+      <c r="L30" s="44"/>
+      <c r="M30" s="7" t="s">
+        <v>640</v>
+      </c>
+      <c r="N30" s="45" t="s">
+        <v>6</v>
+      </c>
+      <c r="O30" s="68" t="s">
+        <v>510</v>
+      </c>
+      <c r="V30" s="70" t="s">
+        <v>206</v>
+      </c>
+      <c r="W30" s="70">
+        <v>4704</v>
+      </c>
+      <c r="X30" s="70" t="s">
+        <v>597</v>
+      </c>
     </row>
     <row r="31" spans="1:24" x14ac:dyDescent="0.2">
       <c r="H31" s="1" t="s">
-        <v>743</v>
-      </c>
-      <c r="I31" s="11"/>
-      <c r="J31" s="1"/>
-      <c r="K31" s="1"/>
+        <v>742</v>
+      </c>
       <c r="L31" s="1"/>
     </row>
     <row r="32" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="I32" s="11"/>
-      <c r="J32" s="1"/>
-      <c r="K32" s="1"/>
       <c r="L32" s="1"/>
     </row>
-    <row r="33" spans="9:18" x14ac:dyDescent="0.2">
-      <c r="I33" s="11"/>
-      <c r="J33" s="1"/>
-      <c r="K33" s="1"/>
+    <row r="33" spans="12:18" x14ac:dyDescent="0.2">
       <c r="L33" s="1"/>
     </row>
-    <row r="34" spans="9:18" x14ac:dyDescent="0.2">
-      <c r="I34" s="11"/>
-      <c r="J34" s="1"/>
-      <c r="K34" s="1"/>
+    <row r="34" spans="12:18" x14ac:dyDescent="0.2">
       <c r="L34" s="1"/>
     </row>
-    <row r="35" spans="9:18" x14ac:dyDescent="0.2">
-      <c r="I35" s="11"/>
-      <c r="J35" s="1"/>
-      <c r="K35" s="1"/>
+    <row r="35" spans="12:18" x14ac:dyDescent="0.2">
       <c r="L35" s="1"/>
     </row>
-    <row r="40" spans="9:18" x14ac:dyDescent="0.2">
-      <c r="R40" s="6"/>
+    <row r="40" spans="12:18" x14ac:dyDescent="0.2">
+      <c r="R40" s="27"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C24" r:id="rId1" xr:uid="{51B5B240-F127-424D-934E-35581681C3C1}"/>
-    <hyperlink ref="K24" r:id="rId2" display="?" xr:uid="{B55DD6F4-6DFA-F748-B417-2D6FE5C2C5B6}"/>
-    <hyperlink ref="N24" r:id="rId3" xr:uid="{6ACA983C-1371-ED47-902A-15D9AD890924}"/>
+    <hyperlink ref="C30" r:id="rId1" xr:uid="{51B5B240-F127-424D-934E-35581681C3C1}"/>
+    <hyperlink ref="K30" r:id="rId2" display="?" xr:uid="{B55DD6F4-6DFA-F748-B417-2D6FE5C2C5B6}"/>
+    <hyperlink ref="N30" r:id="rId3" xr:uid="{6ACA983C-1371-ED47-902A-15D9AD890924}"/>
     <hyperlink ref="C3" r:id="rId4" xr:uid="{909FEFB2-4956-204A-843C-00B985B282CB}"/>
     <hyperlink ref="K3" r:id="rId5" display="https://www.universityofcalifornia.edu/about-us/information-center/doctoral-program" xr:uid="{2D6345EB-9B56-6047-8029-A392A00D013F}"/>
     <hyperlink ref="H3" r:id="rId6" display="Personal History Statement (~1,2p)" xr:uid="{3553C041-D267-DC43-BD94-E0A93A537FD3}"/>
@@ -12788,7 +12940,7 @@
     <hyperlink ref="M13" r:id="rId61" display="GRASP" xr:uid="{DE823A40-C140-DE43-950E-CCA09F47F0EB}"/>
     <hyperlink ref="S4" r:id="rId62" xr:uid="{3107D36A-7816-0540-96C4-74EF2B6CB421}"/>
     <hyperlink ref="Q4" r:id="rId63" xr:uid="{188C7A52-FE43-754F-8376-B52B3291F058}"/>
-    <hyperlink ref="O24" r:id="rId64" xr:uid="{8303D648-D25D-C24E-BEE7-80701D18D5AB}"/>
+    <hyperlink ref="O30" r:id="rId64" xr:uid="{8303D648-D25D-C24E-BEE7-80701D18D5AB}"/>
     <hyperlink ref="R11" r:id="rId65" xr:uid="{C466F216-F9DD-E043-B5E3-FA91388CB9DA}"/>
     <hyperlink ref="O11" r:id="rId66" xr:uid="{9A9F50B7-7E5C-A242-9AA0-8F4A93473724}"/>
     <hyperlink ref="N19" r:id="rId67" xr:uid="{CBE57E7C-0C01-E044-86D1-E1B8FB8205DF}"/>
@@ -12826,7 +12978,7 @@
     <hyperlink ref="P12" r:id="rId99" xr:uid="{9949A074-DDD8-0748-A3D5-D296EE2CB2E6}"/>
     <hyperlink ref="N12" r:id="rId100" xr:uid="{9CA5BC65-45BA-CA4B-BB50-70554955B512}"/>
     <hyperlink ref="H10" r:id="rId101" xr:uid="{68701F73-D566-3C4A-BAB4-5FF42E7B15B1}"/>
-    <hyperlink ref="M24" r:id="rId102" xr:uid="{81606837-51A2-4C4D-8F7C-74672D0A0AE7}"/>
+    <hyperlink ref="M30" r:id="rId102" xr:uid="{81606837-51A2-4C4D-8F7C-74672D0A0AE7}"/>
     <hyperlink ref="M3" r:id="rId103" xr:uid="{4A7FD456-BBDB-5C41-8E50-1899168920A1}"/>
     <hyperlink ref="M4" r:id="rId104" display="IRIM" xr:uid="{07717B9D-4A30-2D46-A24F-29C2EC8A2F57}"/>
     <hyperlink ref="M5" r:id="rId105" xr:uid="{C25FBFE7-937C-674B-8FB8-4203D37F3AFC}"/>
@@ -12859,14 +13011,14 @@
     <hyperlink ref="H9" r:id="rId132" display="Personal Statement (Unlimited)" xr:uid="{71E9B93E-CA71-924E-ABF3-1BF301BAF16A}"/>
     <hyperlink ref="E18" r:id="rId133" display="https://cs.unc.edu/graduate/graduate-admissions/admissions-deadline/" xr:uid="{A8DA038C-62AF-7049-923E-C802B5D0F120}"/>
     <hyperlink ref="C18" r:id="rId134" xr:uid="{1F11307D-180C-7F4E-8F58-3C796024EADC}"/>
-    <hyperlink ref="C2" r:id="rId135" xr:uid="{9BBA89A6-0F3B-DC48-9929-53F346B0AEC8}"/>
-    <hyperlink ref="K2" r:id="rId136" display="?" xr:uid="{44F0BD16-9489-304C-AA7B-73439E846FB2}"/>
-    <hyperlink ref="N2" r:id="rId137" location="people" xr:uid="{8000CF1A-E833-7046-85A6-F8FD94F89DD6}"/>
-    <hyperlink ref="P2" r:id="rId138" xr:uid="{1020D82E-17AD-0843-92AB-4DEFC033D629}"/>
-    <hyperlink ref="O2" r:id="rId139" xr:uid="{47F0EA44-5277-5445-BB7A-BDDCF1050356}"/>
-    <hyperlink ref="Q2" r:id="rId140" xr:uid="{44235266-313A-EB4D-822B-20B3417A492B}"/>
-    <hyperlink ref="R2" r:id="rId141" xr:uid="{0DA4B984-247B-014C-AF10-7B70DD5E6E5B}"/>
-    <hyperlink ref="M2" r:id="rId142" xr:uid="{CF22B631-12A1-DF4D-B5B5-DC93A74172A4}"/>
+    <hyperlink ref="C29" r:id="rId135" xr:uid="{9BBA89A6-0F3B-DC48-9929-53F346B0AEC8}"/>
+    <hyperlink ref="K29" r:id="rId136" display="?" xr:uid="{44F0BD16-9489-304C-AA7B-73439E846FB2}"/>
+    <hyperlink ref="N29" r:id="rId137" location="people" xr:uid="{8000CF1A-E833-7046-85A6-F8FD94F89DD6}"/>
+    <hyperlink ref="P29" r:id="rId138" xr:uid="{1020D82E-17AD-0843-92AB-4DEFC033D629}"/>
+    <hyperlink ref="O29" r:id="rId139" xr:uid="{47F0EA44-5277-5445-BB7A-BDDCF1050356}"/>
+    <hyperlink ref="Q29" r:id="rId140" xr:uid="{44235266-313A-EB4D-822B-20B3417A492B}"/>
+    <hyperlink ref="R29" r:id="rId141" xr:uid="{0DA4B984-247B-014C-AF10-7B70DD5E6E5B}"/>
+    <hyperlink ref="M29" r:id="rId142" xr:uid="{CF22B631-12A1-DF4D-B5B5-DC93A74172A4}"/>
     <hyperlink ref="N5" r:id="rId143" xr:uid="{76506796-C1E0-6349-ABE0-0536ABD45091}"/>
     <hyperlink ref="K8" r:id="rId144" display="12%(36/313)" xr:uid="{B150AADE-A14F-C24C-B2FF-F7650A150E11}"/>
     <hyperlink ref="C8" r:id="rId145" xr:uid="{BEB53160-CC16-4B4F-8683-4043A3679F0E}"/>
@@ -12901,6 +13053,8 @@
     <hyperlink ref="O15" r:id="rId174" xr:uid="{1C8BE2D9-25D8-7040-AFBB-870B90C39D41}"/>
     <hyperlink ref="P11" r:id="rId175" xr:uid="{5A0E2DC6-7112-CB42-8B13-0D714E7EE698}"/>
     <hyperlink ref="Q11" r:id="rId176" xr:uid="{BC88C10D-785F-534A-B349-B2DA4E7086B9}"/>
+    <hyperlink ref="J5" r:id="rId177" display="Accept LoR after deadline" xr:uid="{240597F5-DBD6-B24D-A770-7F680D569E5B}"/>
+    <hyperlink ref="C2" r:id="rId178" xr:uid="{89DD44D2-039D-2D4B-BF53-164442E02001}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>